<commit_message>
Fix supplementary tables S2-S5
- S2: Added Community_label for 14 isolated WHO priority genes
- S3: Fixed mcr-4.7 R2=0.000; p-values floored at 0.0001
- S4: Fixed arr and mcr-4.7 KW_H=0, P=1.0; p-values floored at 0.0001
- S5: Labeled bnlearn-only edges Jaccard as NA (bnlearn only)
</commit_message>
<xml_diff>
--- a/results/supplementary/tables_submission/TableS5_network_consensus_edges.xlsx
+++ b/results/supplementary/tables_submission/TableS5_network_consensus_edges.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TableS5_network_consensus_edges" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,16 +40,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E4057"/>
+        <bgColor rgb="002E4057"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,11 +70,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,13 +441,13 @@
   <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,10 +503,8 @@
           <t>0.4851</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+      <c r="D2" s="2" t="n">
+        <v>0.998</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -542,13 +535,11 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>0.4570</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+          <t>0.457</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.998</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
@@ -582,10 +573,8 @@
           <t>0.3276</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="D4" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -616,13 +605,11 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>0.4270</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
@@ -656,10 +643,8 @@
           <t>0.3097</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>0.8789</t>
-        </is>
+      <c r="D6" s="2" t="n">
+        <v>0.8789</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -693,10 +678,8 @@
           <t>0.4325</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="D7" s="3" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
@@ -730,10 +713,8 @@
           <t>0.6519</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>0.8574</t>
-        </is>
+      <c r="D8" s="2" t="n">
+        <v>0.8574000000000001</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -767,10 +748,8 @@
           <t>0.9864</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
@@ -804,10 +783,8 @@
           <t>0.8722</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>0.9375</t>
-        </is>
+      <c r="D10" s="2" t="n">
+        <v>0.9375</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -841,10 +818,8 @@
           <t>0.4786</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D11" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -878,10 +853,8 @@
           <t>0.5561</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>0.8652</t>
-        </is>
+      <c r="D12" s="2" t="n">
+        <v>0.8652</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -915,10 +888,8 @@
           <t>0.8808</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+      <c r="D13" s="3" t="n">
+        <v>0.998</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
@@ -952,10 +923,8 @@
           <t>0.3592</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>0.9453</t>
-        </is>
+      <c r="D14" s="2" t="n">
+        <v>0.9453</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -989,10 +958,8 @@
           <t>0.3385</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>0.9824</t>
-        </is>
+      <c r="D15" s="3" t="n">
+        <v>0.9824000000000001</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
@@ -1026,10 +993,8 @@
           <t>0.5867</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>0.9922</t>
-        </is>
+      <c r="D16" s="2" t="n">
+        <v>0.9922</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -1063,10 +1028,8 @@
           <t>0.3729</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D17" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
@@ -1100,10 +1063,8 @@
           <t>0.5005</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D18" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -1134,13 +1095,11 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>0.3440</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>0.9863</t>
-        </is>
+          <t>0.344</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.9863</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
@@ -1174,10 +1133,8 @@
           <t>0.6114</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>0.9160</t>
-        </is>
+      <c r="D20" s="2" t="n">
+        <v>0.916</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -1211,10 +1168,8 @@
           <t>0.6296</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>0.8652</t>
-        </is>
+      <c r="D21" s="3" t="n">
+        <v>0.8652</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
@@ -1248,10 +1203,8 @@
           <t>0.4144</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D22" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -1282,13 +1235,11 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>0.4050</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+          <t>0.405</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
@@ -1322,10 +1273,8 @@
           <t>0.8418</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>0.9844</t>
-        </is>
+      <c r="D24" s="2" t="n">
+        <v>0.9844000000000001</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -1359,10 +1308,8 @@
           <t>0.7161</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>0.9492</t>
-        </is>
+      <c r="D25" s="3" t="n">
+        <v>0.9492</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
@@ -1396,10 +1343,8 @@
           <t>0.9475</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D26" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -1433,10 +1378,8 @@
           <t>0.7575</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>0.9102</t>
-        </is>
+      <c r="D27" s="3" t="n">
+        <v>0.9102</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
@@ -1470,10 +1413,8 @@
           <t>0.9788</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D28" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -1504,13 +1445,11 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>0.8290</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+          <t>0.829</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
@@ -1544,10 +1483,8 @@
           <t>0.6881</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>0.8516</t>
-        </is>
+      <c r="D30" s="2" t="n">
+        <v>0.8516</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -1581,10 +1518,8 @@
           <t>0.7039</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>0.9473</t>
-        </is>
+      <c r="D31" s="3" t="n">
+        <v>0.9473</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
@@ -1618,10 +1553,8 @@
           <t>0.3273</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D32" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -1655,10 +1588,8 @@
           <t>0.7627</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D33" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
@@ -1692,10 +1623,8 @@
           <t>0.4684</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D34" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
@@ -1729,10 +1658,8 @@
           <t>0.4545</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>0.8965</t>
-        </is>
+      <c r="D35" s="3" t="n">
+        <v>0.8965</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
@@ -1766,10 +1693,8 @@
           <t>0.5456</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D36" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -1803,10 +1728,8 @@
           <t>0.3298</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>0.9883</t>
-        </is>
+      <c r="D37" s="3" t="n">
+        <v>0.9883</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
@@ -1837,13 +1760,11 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>0.7160</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+          <t>0.716</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1798,8 @@
           <t>0.6735</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D39" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
@@ -1911,13 +1830,11 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>0.5180</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+          <t>0.518</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -1951,10 +1868,8 @@
           <t>0.6286</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="D41" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
@@ -1988,10 +1903,8 @@
           <t>0.4947</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>0.9766</t>
-        </is>
+      <c r="D42" s="2" t="n">
+        <v>0.9766</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -2020,11 +1933,13 @@
           <t>aph(3')</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>0.9805</t>
-        </is>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>0.9805</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
@@ -2053,11 +1968,13 @@
           <t>blaoxa_235like</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>0.8594</t>
-        </is>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0.8594000000000001</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
@@ -2086,11 +2003,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
@@ -2119,11 +2038,13 @@
           <t>ftsi</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>0.9688</t>
-        </is>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0.9688</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
@@ -2152,11 +2073,13 @@
           <t>adec</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0.998</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
@@ -2185,11 +2108,13 @@
           <t>aph(3')</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
@@ -2218,11 +2143,13 @@
           <t>ftsi</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>0.9863</t>
-        </is>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0.9863</v>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
@@ -2251,11 +2178,13 @@
           <t>tet(b)</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>0.9785</t>
-        </is>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>0.9785</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
@@ -2284,11 +2213,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
@@ -2317,11 +2248,13 @@
           <t>aada</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>0.9609</t>
-        </is>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0.9609</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
@@ -2350,11 +2283,13 @@
           <t>adec</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>0.9941</t>
-        </is>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>0.9941</v>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
@@ -2383,11 +2318,13 @@
           <t>aph(3')</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
@@ -2416,11 +2353,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>0.9277</t>
-        </is>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>0.9277</v>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
@@ -2449,11 +2388,13 @@
           <t>catb</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
@@ -2482,11 +2423,13 @@
           <t>ftsi</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>0.8984</t>
-        </is>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>0.8984</v>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
@@ -2515,11 +2458,13 @@
           <t>qacedelta</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>0.9043</t>
-        </is>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>0.9043</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
@@ -2548,11 +2493,13 @@
           <t>sul</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>0.9492</t>
-        </is>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>0.9492</v>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
@@ -2581,11 +2528,13 @@
           <t>tet(b)</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>0.998</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
@@ -2614,11 +2563,13 @@
           <t>aac(6')</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr"/>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>0.9102</t>
-        </is>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>0.9102</v>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
@@ -2647,11 +2598,13 @@
           <t>blandm</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
@@ -2680,11 +2633,13 @@
           <t>ftsi</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr"/>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>0.9727</t>
-        </is>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>0.9727</v>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
@@ -2713,11 +2668,13 @@
           <t>qacedelta</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr"/>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>0.9258</t>
-        </is>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>0.9258</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
@@ -2746,11 +2703,13 @@
           <t>tet(b)</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr"/>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>0.9121</t>
-        </is>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>0.9121</v>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
@@ -2779,11 +2738,13 @@
           <t>aph(3')</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>0.9980</t>
-        </is>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0.998</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
@@ -2812,11 +2773,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr"/>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
@@ -2845,11 +2808,13 @@
           <t>blaoxa_235like</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr"/>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>0.9551</t>
-        </is>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>0.9550999999999999</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
@@ -2878,11 +2843,13 @@
           <t>blaoxa_23like</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr"/>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
@@ -2911,11 +2878,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr"/>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>0.9961</t>
-        </is>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0.9961</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
@@ -2944,11 +2913,13 @@
           <t>blaoxa_23like</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr"/>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>0.9922</t>
-        </is>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>0.9922</v>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
@@ -2977,11 +2948,13 @@
           <t>parc</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr"/>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>0.8730</t>
-        </is>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>0.873</v>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
@@ -3010,11 +2983,13 @@
           <t>aac(3)</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr"/>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>0.9141</t>
-        </is>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>0.9141</v>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
@@ -3043,11 +3018,13 @@
           <t>aac(6')</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr"/>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>0.9648</t>
-        </is>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>0.9648</v>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
@@ -3076,11 +3053,13 @@
           <t>aada</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr"/>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
@@ -3109,11 +3088,13 @@
           <t>adec</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr"/>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
@@ -3142,11 +3123,13 @@
           <t>aph(3'')</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr"/>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>0.9902</t>
-        </is>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>0.9902</v>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
@@ -3175,11 +3158,13 @@
           <t>aph(6)</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>0.9121</t>
-        </is>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0.9121</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
@@ -3208,11 +3193,13 @@
           <t>arma</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr"/>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>0.9238</t>
-        </is>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>0.9238</v>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
@@ -3241,11 +3228,13 @@
           <t>catb</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr"/>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
@@ -3274,11 +3263,13 @@
           <t>parc</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr"/>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>0.9805</t>
-        </is>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>0.9805</v>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
@@ -3307,11 +3298,13 @@
           <t>qacedelta</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr"/>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
@@ -3340,11 +3333,13 @@
           <t>blatem</t>
         </is>
       </c>
-      <c r="C83" s="3" t="inlineStr"/>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>0.9609</t>
-        </is>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>NA (bnlearn only)</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>0.9609</v>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>

</xml_diff>